<commit_message>
Versão final do gerador de PDF
</commit_message>
<xml_diff>
--- a/Exemplo de excel.xlsx
+++ b/Exemplo de excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29926"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Suporte Plano\Desktop\PDF_redirecionavel_JS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\PDF_Interativo_JS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACDE093E-3F96-4CA3-9015-27543EEC71B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04579E7-66C6-4602-96BB-F8A48767B2BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5D8282FC-8ADA-4895-8575-968A37F3B1B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5D8282FC-8ADA-4895-8575-968A37F3B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="6">
   <si>
     <t>Item 1</t>
   </si>
@@ -98,9 +98,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -138,7 +138,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -244,7 +244,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -386,7 +386,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -395,7 +395,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D928AB7-CCB2-4B9C-8EC1-22E89FFE24A1}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -441,6 +441,86 @@
         <v>25.9</v>
       </c>
     </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15">
+        <v>25.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>